<commit_message>
Update finals: brief email, PRD strategic note, Excel 8-field corrections
- email-printify.html: rewritten as short intro cover email (no methodology tables)
- prd-v5.html: added strategic timeline note (not a 6-month project framing)
- Printify_Leather_PRD_Workbook.xlsx: updated with 8 schema fields, Amazon BSR 8,365, TAM $54.26B, W16 demand chart point

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/finals/Printify_Leather_PRD_Workbook.xlsx
+++ b/output/finals/Printify_Leather_PRD_Workbook.xlsx
@@ -2869,7 +2869,7 @@
       </c>
       <c r="G6" s="42" t="inlineStr">
         <is>
-          <t>Printify apparel onboarding benchmark: complex forms without AI assist average 3–5 days. AI field-assist pre-fills 7 schema fields → estimated 70% reduction. Target 24h is achievable with assisted flow.</t>
+          <t>Printify apparel onboarding benchmark: complex forms without AI assist average 3–5 days. AI field-assist pre-fills 8 schema fields → estimated 70% reduction. Target 24h is achievable with assisted flow.</t>
         </is>
       </c>
       <c r="H6" s="43" t="inlineStr">
@@ -3747,7 +3747,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3882,7 +3882,7 @@
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>&gt; 8,000 units / month</t>
+          <t>BULLIANT wallet — 8,365 units / month (BSR rank)</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
@@ -3897,7 +3897,7 @@
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>Single top SKU proxy — not category average</t>
+          <t>Single mature listing proxy — new POD SKU enters at 5–20/mo</t>
         </is>
       </c>
     </row>
@@ -3914,7 +3914,7 @@
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>$41B total / ~$2B POD-addressable (estimate)</t>
+          <t>$54.26B total · 6.7% CAGR · custom/POD ~$2B addressable (est.)</t>
         </is>
       </c>
       <c r="D8" s="18" t="inlineStr">
@@ -4309,64 +4309,80 @@
     <row r="31" customHeight="1">
       <c r="A31" t="inlineStr">
         <is>
-          <t>M0 Launch</t>
+          <t>W16 Shopify G1</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C31" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D31" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="32" customHeight="1">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Month 1</t>
+          <t>M0 Launch</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="D32" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33" customHeight="1">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Month 2 ◆</t>
+          <t>Month 1</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C33" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="D33" t="n">
-        <v>50</v>
+        <v>35</v>
       </c>
     </row>
     <row r="34" customHeight="1">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Month 3</t>
+          <t>Month 2 ◆</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>8</v>
       </c>
       <c r="C34" t="n">
+        <v>22</v>
+      </c>
+      <c r="D34" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="35" customHeight="1">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Month 3</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>8</v>
+      </c>
+      <c r="C35" t="n">
         <v>25</v>
       </c>
-      <c r="D34" t="n">
+      <c r="D35" t="n">
         <v>60</v>
       </c>
     </row>
@@ -4946,7 +4962,7 @@
       </c>
       <c r="E29" s="10" t="inlineStr">
         <is>
-          <t>7 blueprint schema fields · MAT-001 FTC AI classifier · laser_engraving + debossing enum API updates · audit log</t>
+          <t>8 blueprint schema fields · MAT-001 FTC AI classifier · laser_engraving + debossing enum API updates · audit log</t>
         </is>
       </c>
       <c r="F29" s="10" t="inlineStr">
@@ -5905,7 +5921,7 @@
       </c>
       <c r="C7" s="98" t="inlineStr">
         <is>
-          <t>✅ 7 fields</t>
+          <t>✅ 8 fields</t>
         </is>
       </c>
       <c r="D7" s="93" t="inlineStr">
@@ -6782,7 +6798,7 @@
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>7 schema fields (material_tier, tannage_method, origin_country, finish_type, thickness_mm, prop_65_compliant, laser_engraving_area) · MAT-001 AI classifier · laser_engraving + debossing API enums</t>
+          <t>8 schema fields (leather_grade, tanning_method, finish_type, hide_thickness_mm, hide_origin, grain_correction, compliance_cert, eco_claims) · MAT-001 AI classifier · laser_engraving + debossing API enums</t>
         </is>
       </c>
       <c r="F7" s="10" t="inlineStr">
@@ -6815,7 +6831,7 @@
       </c>
       <c r="E8" s="57" t="inlineStr">
         <is>
-          <t>Static leather texture mockup engine (3 textures/tier · assets locked W9D1) · Decorator portal (7 fields, plain-language) · AI field-assist agent · MAT-001 scoring UX · 5 Decorators complete onboarding</t>
+          <t>Static leather texture mockup engine (3 textures/tier · assets locked W9D1) · Decorator portal (8 fields, plain-language) · AI field-assist agent · MAT-001 scoring UX · 5 Decorators complete onboarding</t>
         </is>
       </c>
       <c r="F8" s="57" t="inlineStr">

</xml_diff>